<commit_message>
Final test report for PA5
</commit_message>
<xml_diff>
--- a/docs/test/test-plans/Test case Dashboard.xlsx
+++ b/docs/test/test-plans/Test case Dashboard.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="211">
   <si>
     <t xml:space="preserve">Project: Recall AI</t>
   </si>
@@ -2163,8 +2163,8 @@
       <c r="F16" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="G16" s="12" t="n">
-        <v>3</v>
+      <c r="G16" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>42</v>

</xml_diff>